<commit_message>
Clean up untracked files and update test workbook
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -908,7 +908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1371,6 +1371,52 @@
         <is>
           <t>Attributed Revenue - Raw Meta Spend = Profit</t>
         </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>14. Spend Attribution Disconnect</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>14. Spend Attribution Disconnect</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix verification crash and make campaign normalization universally robust
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -908,7 +908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1393,29 +1393,6 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>14. Spend Attribution Disconnect</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Amount Spent KeyError, enforce canonical spend, fix tests
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -14,13 +14,7 @@
     <sheet name="5. 🎨 Ad Creative Summary" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="6. 📍 Placement Summary" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="7. 🏦 Ad Account Comparison" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="8. 💰 Free vs Paid Funnel" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="9. 🚨 Zero-ROI Waste Report" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="10. ❓ Unattributed Sales" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="11. 🔁 Old Leads (Separate)" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="12. 💳 Spend Reference" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="13. ✅ Verification" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="14. 🚫 Excluded Sales" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="8. 🚨 Zero-ROI Waste Report" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -588,7 +582,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -608,7 +602,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -648,7 +642,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -687,8 +681,10 @@
           <t>Per Sale Value</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>8999</v>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -697,8 +693,10 @@
           <t>Attributed Per Sale Value</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>8999</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -836,585 +834,6 @@
           <t>N/A</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Check Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Expected</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Actual</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Difference</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Explanation</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1. All Sales row count</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Matches valid input sales rows after exclusions</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2. Summary Sales Match</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>C:0, AS:0, AD:0</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Campaign/AdSet/Ad Sales totals must equal Attributed Sales (0). 0 unattributed sale(s) correctly excluded from summaries.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>3. Summary Revenue Match</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>C:0.0, AS:0.0, AD:0.0</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Campaign/AdSet/Ad Revenue totals must equal Attributed Revenue (unattributed revenue excluded)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>4. Spend Invariant</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Attributed Spend + Unallocated Spend must exactly equal Total Windowed Meta Spend</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>5. Summary Spend Reconcile</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>C:0.0, AS:0.0, AD:0.0</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Summary spend totals reconcile with Total Windowed Meta Spend</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>6. Duplicate Sales Email</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Report duplicate sales-email count</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>7. Unattributed Rate</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Warn if &gt; 10% unattributed. Current: 0.0% (0 sales)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>8. Funnel Leads Match</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Every lead counted exactly once in funnel summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>9. Reg Fee Revenue Match</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Registration fee revenue equals qualifying fees in Leads sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>10. Derived Sale Dates</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Count of sales using derived dates (Lead Reg/Start Date/Custom)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>11. Assumed Payment Status</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Count of sales explicitly assuming successful payment</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>12. Fallback Order Amounts</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Count of sales using fallback price due to missing order amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>13. Unresolved/Missing Sales Dates</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Count of sales that still lack a valid sale date</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>INV. Revenue Formula</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Attributed + Unattributed = Total Revenue</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>INV. Spend Formula</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Attributed + Unallocated = Raw Meta Spend</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>INV. Profit Formula</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Attributed Revenue - Raw Meta Spend = Profit</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>14. Spend Attribution Disconnect</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1505,82 +924,100 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="5" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
     <col width="5" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>camp_norm</t>
+          <t>Campaign Name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Spend</t>
+          <t>Total Leads</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Leads</t>
+          <t>Total Sales</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Attributed Sales</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Raw Meta Spend</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Spend / Cost</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>CPL</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Conversion Rate %</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>CAC</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ROAS</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ROI</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Conversion Rate</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Profit</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>ROAS</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>ROI %</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>CAC</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Profitable?</t>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Price Per Sale</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Funnel Type</t>
         </is>
       </c>
     </row>
@@ -1949,66 +1386,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Funnel Stage</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Total Leads</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Paid Leads</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Unpaid Leads</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Include all final acceptance test scripts and utilities
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -12,9 +12,6 @@
     <sheet name="3. 📢 Campaign Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="4. 🎯 Ad Set Summary" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5. 🎨 Ad Creative Summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="6. 📍 Placement Summary" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="7. 🏦 Ad Account Comparison" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="8. 🚨 Zero-ROI Waste Report" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -846,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -858,7 +855,6 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -905,11 +901,6 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>ad_norm</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>placement_norm</t>
         </is>
       </c>
     </row>
@@ -924,100 +915,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="5" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
     <col width="5" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Campaign Name</t>
+          <t>camp_norm</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Total Leads</t>
+          <t>Spend</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Total Sales</t>
+          <t>Leads</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Attributed Sales</t>
+          <t>CPL</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Total Revenue</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Raw Meta Spend</t>
+          <t>Conversion Rate %</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Spend / Cost</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>CPL</t>
+          <t>Profit</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>ROAS</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ROI %</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>CAC</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>ROAS</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>ROI</t>
-        </is>
-      </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Conversion Rate</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Profit</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Price Per Sale</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Funnel Type</t>
+          <t>Profitable?</t>
         </is>
       </c>
     </row>
@@ -1222,180 +1195,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="5" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>camp_norm</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>placement_norm</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Spend</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Leads</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>CPL</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Conversion Rate %</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Profit</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>ROAS</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>ROI %</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>CAC</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Profitable?</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Raw Meta Spend</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Attributed Spend</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Unallocated Spend</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>